<commit_message>
feat: add form selection, image fetcher, and updated prompts/templates
</commit_message>
<xml_diff>
--- a/Form.xlsx
+++ b/Form.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lut.sharepoint.com/sites/o365BK10A6300EngineeringDesign-Coursematerials/Shared Documents/Course materials/2025-2026/2_Exercises/Exercise 1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mdsazzadurrahman/Documents/ai-agent-for-filling-detasheet/Untitled/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{388EB0FF-B0CF-463D-A921-466F2BCE0BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A51224B7-ADE4-453C-889C-26531E0D7C9D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF947ED1-3B9E-1D4C-B3CE-CC9B5A9D5934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5520" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{DD70C75C-9463-475E-BB7C-8F1DF3114433}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17260" activeTab="1" xr2:uid="{DD70C75C-9463-475E-BB7C-8F1DF3114433}"/>
   </bookViews>
   <sheets>
     <sheet name="EBOM" sheetId="20" r:id="rId1"/>
@@ -544,7 +544,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1389,6 +1389,249 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="41" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="21" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="22" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="19" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="25" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="25" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="26" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1466,249 +1709,6 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="27" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="25" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="25" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="26" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="21" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="22" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="19" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="41" xfId="8" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -1803,54 +1803,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>285198</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>82550</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>280147</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>159998</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CCF67D76-EEC6-4A5E-B844-D26F406B407F}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:srcRect l="4930" t="5868" r="4296" b="9032"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5607992" y="855756"/>
-          <a:ext cx="1810302" cy="1433360"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2151,477 +2103,477 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A24E4985-ACB0-4321-964C-D19C2C2FB620}">
   <dimension ref="A1:O21"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="2"/>
-    <col min="2" max="2" width="18.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="9.1640625" style="2"/>
+    <col min="2" max="2" width="18.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" style="2" customWidth="1"/>
     <col min="4" max="4" width="17" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="20.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" style="1" customWidth="1"/>
     <col min="8" max="8" width="70" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="2"/>
+    <col min="9" max="9" width="12.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.1640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="30" customHeight="1">
-      <c r="A1" s="113" t="s">
+    <row r="1" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="113" t="s">
+      <c r="B1" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="113" t="s">
+      <c r="C1" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="113" t="s">
+      <c r="D1" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="113" t="s">
+      <c r="E1" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="113" t="s">
+      <c r="F1" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="114" t="s">
+      <c r="G1" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="114" t="s">
+      <c r="H1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="115" t="s">
+      <c r="I1" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="115" t="s">
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="N1" s="116"/>
-      <c r="O1" s="117"/>
-    </row>
-    <row r="2" spans="1:15">
-      <c r="A2" s="118"/>
-      <c r="B2" s="118"/>
-      <c r="C2" s="118"/>
-      <c r="D2" s="118"/>
-      <c r="E2" s="118"/>
-      <c r="F2" s="118"/>
-      <c r="G2" s="119"/>
-      <c r="H2" s="119"/>
-      <c r="I2" s="120" t="s">
+      <c r="N1" s="28"/>
+      <c r="O1" s="29"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="120" t="s">
+      <c r="J2" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="K2" s="120" t="s">
+      <c r="K2" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="120" t="s">
+      <c r="L2" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="121" t="s">
+      <c r="M2" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="N2" s="121" t="s">
+      <c r="N2" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="O2" s="121" t="s">
+      <c r="O2" s="22" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:15" s="3" customFormat="1">
-      <c r="A3" s="108" t="s">
+    <row r="3" spans="1:15" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="109" t="s">
+      <c r="B3" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="109" t="s">
+      <c r="C3" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="109" t="s">
+      <c r="D3" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="109" t="s">
+      <c r="E3" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="110" t="s">
+      <c r="F3" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="G3" s="111" t="s">
+      <c r="G3" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="109" t="s">
+      <c r="H3" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="I3" s="108"/>
-      <c r="J3" s="108"/>
-      <c r="K3" s="108"/>
-      <c r="L3" s="108"/>
-      <c r="M3" s="108"/>
-      <c r="N3" s="108"/>
-      <c r="O3" s="108"/>
-    </row>
-    <row r="4" spans="1:15">
-      <c r="A4" s="107" t="s">
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A4" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="107"/>
-      <c r="C4" s="107"/>
-      <c r="D4" s="107"/>
-      <c r="E4" s="107"/>
-      <c r="F4" s="107"/>
-      <c r="G4" s="112"/>
-      <c r="H4" s="107"/>
-      <c r="I4" s="107"/>
-      <c r="J4" s="107"/>
-      <c r="K4" s="107"/>
-      <c r="L4" s="107"/>
-      <c r="M4" s="107"/>
-      <c r="N4" s="107"/>
-      <c r="O4" s="107"/>
-    </row>
-    <row r="5" spans="1:15">
-      <c r="A5" s="107" t="s">
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="107"/>
-      <c r="C5" s="107"/>
-      <c r="D5" s="107"/>
-      <c r="E5" s="107"/>
-      <c r="F5" s="107"/>
-      <c r="G5" s="112"/>
-      <c r="H5" s="107"/>
-      <c r="I5" s="107"/>
-      <c r="J5" s="107"/>
-      <c r="K5" s="107"/>
-      <c r="L5" s="107"/>
-      <c r="M5" s="107"/>
-      <c r="N5" s="107"/>
-      <c r="O5" s="107"/>
-    </row>
-    <row r="6" spans="1:15">
-      <c r="A6" s="107" t="s">
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A6" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="107"/>
-      <c r="C6" s="107"/>
-      <c r="D6" s="107"/>
-      <c r="E6" s="107"/>
-      <c r="F6" s="107"/>
-      <c r="G6" s="112"/>
-      <c r="H6" s="107"/>
-      <c r="I6" s="107"/>
-      <c r="J6" s="107"/>
-      <c r="K6" s="107"/>
-      <c r="L6" s="107"/>
-      <c r="M6" s="107"/>
-      <c r="N6" s="107"/>
-      <c r="O6" s="107"/>
-    </row>
-    <row r="7" spans="1:15">
-      <c r="A7" s="107" t="s">
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="15"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="15"/>
+      <c r="O6" s="15"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A7" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="107"/>
-      <c r="C7" s="107"/>
-      <c r="D7" s="107"/>
-      <c r="E7" s="107"/>
-      <c r="F7" s="107"/>
-      <c r="G7" s="112"/>
-      <c r="H7" s="107"/>
-      <c r="I7" s="107"/>
-      <c r="J7" s="107"/>
-      <c r="K7" s="107"/>
-      <c r="L7" s="107"/>
-      <c r="M7" s="107"/>
-      <c r="N7" s="107"/>
-      <c r="O7" s="107"/>
-    </row>
-    <row r="8" spans="1:15">
-      <c r="A8" s="107" t="s">
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="15"/>
+      <c r="K7" s="15"/>
+      <c r="L7" s="15"/>
+      <c r="M7" s="15"/>
+      <c r="N7" s="15"/>
+      <c r="O7" s="15"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A8" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="107"/>
-      <c r="C8" s="107"/>
-      <c r="D8" s="107"/>
-      <c r="E8" s="107"/>
-      <c r="F8" s="107"/>
-      <c r="G8" s="112"/>
-      <c r="H8" s="107"/>
-      <c r="I8" s="107"/>
-      <c r="J8" s="107"/>
-      <c r="K8" s="107"/>
-      <c r="L8" s="107"/>
-      <c r="M8" s="107"/>
-      <c r="N8" s="107"/>
-      <c r="O8" s="107"/>
-    </row>
-    <row r="9" spans="1:15">
-      <c r="A9" s="107" t="s">
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="15"/>
+      <c r="O8" s="15"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A9" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="107"/>
-      <c r="C9" s="107"/>
-      <c r="D9" s="107"/>
-      <c r="E9" s="107"/>
-      <c r="F9" s="107"/>
-      <c r="G9" s="112"/>
-      <c r="H9" s="107"/>
-      <c r="I9" s="107"/>
-      <c r="J9" s="107"/>
-      <c r="K9" s="107"/>
-      <c r="L9" s="107"/>
-      <c r="M9" s="107"/>
-      <c r="N9" s="107"/>
-      <c r="O9" s="107"/>
-    </row>
-    <row r="10" spans="1:15">
-      <c r="A10" s="107" t="s">
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15"/>
+      <c r="M9" s="15"/>
+      <c r="N9" s="15"/>
+      <c r="O9" s="15"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A10" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="107"/>
-      <c r="C10" s="107"/>
-      <c r="D10" s="107"/>
-      <c r="E10" s="107"/>
-      <c r="F10" s="107"/>
-      <c r="G10" s="112"/>
-      <c r="H10" s="107"/>
-      <c r="I10" s="107"/>
-      <c r="J10" s="107"/>
-      <c r="K10" s="107"/>
-      <c r="L10" s="107"/>
-      <c r="M10" s="107"/>
-      <c r="N10" s="107"/>
-      <c r="O10" s="107"/>
-    </row>
-    <row r="11" spans="1:15">
-      <c r="A11" s="107" t="s">
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="15"/>
+      <c r="M10" s="15"/>
+      <c r="N10" s="15"/>
+      <c r="O10" s="15"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A11" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="107"/>
-      <c r="C11" s="107"/>
-      <c r="D11" s="107"/>
-      <c r="E11" s="107"/>
-      <c r="F11" s="107"/>
-      <c r="G11" s="112"/>
-      <c r="H11" s="107"/>
-      <c r="I11" s="107"/>
-      <c r="J11" s="107"/>
-      <c r="K11" s="107"/>
-      <c r="L11" s="107"/>
-      <c r="M11" s="107"/>
-      <c r="N11" s="107"/>
-      <c r="O11" s="107"/>
-    </row>
-    <row r="12" spans="1:15">
-      <c r="A12" s="107" t="s">
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
+      <c r="L11" s="15"/>
+      <c r="M11" s="15"/>
+      <c r="N11" s="15"/>
+      <c r="O11" s="15"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A12" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="107"/>
-      <c r="C12" s="107"/>
-      <c r="D12" s="107"/>
-      <c r="E12" s="107"/>
-      <c r="F12" s="107"/>
-      <c r="G12" s="112"/>
-      <c r="H12" s="107"/>
-      <c r="I12" s="107"/>
-      <c r="J12" s="107"/>
-      <c r="K12" s="107"/>
-      <c r="L12" s="107"/>
-      <c r="M12" s="107"/>
-      <c r="N12" s="107"/>
-      <c r="O12" s="107"/>
-    </row>
-    <row r="13" spans="1:15">
-      <c r="A13" s="107" t="s">
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15"/>
+      <c r="L12" s="15"/>
+      <c r="M12" s="15"/>
+      <c r="N12" s="15"/>
+      <c r="O12" s="15"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A13" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="107"/>
-      <c r="C13" s="107"/>
-      <c r="D13" s="107"/>
-      <c r="E13" s="107"/>
-      <c r="F13" s="107"/>
-      <c r="G13" s="112"/>
-      <c r="H13" s="107"/>
-      <c r="I13" s="107"/>
-      <c r="J13" s="107"/>
-      <c r="K13" s="107"/>
-      <c r="L13" s="107"/>
-      <c r="M13" s="107"/>
-      <c r="N13" s="107"/>
-      <c r="O13" s="107"/>
-    </row>
-    <row r="14" spans="1:15">
-      <c r="A14" s="107" t="s">
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="15"/>
+      <c r="L13" s="15"/>
+      <c r="M13" s="15"/>
+      <c r="N13" s="15"/>
+      <c r="O13" s="15"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A14" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B14" s="107"/>
-      <c r="C14" s="107"/>
-      <c r="D14" s="107"/>
-      <c r="E14" s="107"/>
-      <c r="F14" s="107"/>
-      <c r="G14" s="112"/>
-      <c r="H14" s="107"/>
-      <c r="I14" s="107"/>
-      <c r="J14" s="107"/>
-      <c r="K14" s="107"/>
-      <c r="L14" s="107"/>
-      <c r="M14" s="107"/>
-      <c r="N14" s="107"/>
-      <c r="O14" s="107"/>
-    </row>
-    <row r="15" spans="1:15">
-      <c r="A15" s="107" t="s">
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="15"/>
+      <c r="L14" s="15"/>
+      <c r="M14" s="15"/>
+      <c r="N14" s="15"/>
+      <c r="O14" s="15"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A15" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="107"/>
-      <c r="C15" s="107"/>
-      <c r="D15" s="107"/>
-      <c r="E15" s="107"/>
-      <c r="F15" s="107"/>
-      <c r="G15" s="112"/>
-      <c r="H15" s="107"/>
-      <c r="I15" s="107"/>
-      <c r="J15" s="107"/>
-      <c r="K15" s="107"/>
-      <c r="L15" s="107"/>
-      <c r="M15" s="107"/>
-      <c r="N15" s="107"/>
-      <c r="O15" s="107"/>
-    </row>
-    <row r="16" spans="1:15">
-      <c r="A16" s="107" t="s">
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="15"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="15"/>
+      <c r="L15" s="15"/>
+      <c r="M15" s="15"/>
+      <c r="N15" s="15"/>
+      <c r="O15" s="15"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A16" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="107"/>
-      <c r="C16" s="107"/>
-      <c r="D16" s="107"/>
-      <c r="E16" s="107"/>
-      <c r="F16" s="107"/>
-      <c r="G16" s="112"/>
-      <c r="H16" s="107"/>
-      <c r="I16" s="107"/>
-      <c r="J16" s="107"/>
-      <c r="K16" s="107"/>
-      <c r="L16" s="107"/>
-      <c r="M16" s="107"/>
-      <c r="N16" s="107"/>
-      <c r="O16" s="107"/>
-    </row>
-    <row r="17" spans="1:15">
-      <c r="A17" s="107" t="s">
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="15"/>
+      <c r="K16" s="15"/>
+      <c r="L16" s="15"/>
+      <c r="M16" s="15"/>
+      <c r="N16" s="15"/>
+      <c r="O16" s="15"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A17" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="107"/>
-      <c r="C17" s="107"/>
-      <c r="D17" s="107"/>
-      <c r="E17" s="107"/>
-      <c r="F17" s="107"/>
-      <c r="G17" s="112"/>
-      <c r="H17" s="107"/>
-      <c r="I17" s="107"/>
-      <c r="J17" s="107"/>
-      <c r="K17" s="107"/>
-      <c r="L17" s="107"/>
-      <c r="M17" s="107"/>
-      <c r="N17" s="107"/>
-      <c r="O17" s="107"/>
-    </row>
-    <row r="18" spans="1:15">
-      <c r="A18" s="107" t="s">
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="15"/>
+      <c r="I17" s="15"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="15"/>
+      <c r="L17" s="15"/>
+      <c r="M17" s="15"/>
+      <c r="N17" s="15"/>
+      <c r="O17" s="15"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A18" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="107"/>
-      <c r="C18" s="107"/>
-      <c r="D18" s="107"/>
-      <c r="E18" s="107"/>
-      <c r="F18" s="107"/>
-      <c r="G18" s="112"/>
-      <c r="H18" s="107"/>
-      <c r="I18" s="107"/>
-      <c r="J18" s="107"/>
-      <c r="K18" s="107"/>
-      <c r="L18" s="107"/>
-      <c r="M18" s="107"/>
-      <c r="N18" s="107"/>
-      <c r="O18" s="107"/>
-    </row>
-    <row r="19" spans="1:15">
-      <c r="A19" s="107" t="s">
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="20"/>
+      <c r="H18" s="15"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="15"/>
+      <c r="L18" s="15"/>
+      <c r="M18" s="15"/>
+      <c r="N18" s="15"/>
+      <c r="O18" s="15"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A19" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="107"/>
-      <c r="C19" s="107"/>
-      <c r="D19" s="107"/>
-      <c r="E19" s="107"/>
-      <c r="F19" s="107"/>
-      <c r="G19" s="112"/>
-      <c r="H19" s="107"/>
-      <c r="I19" s="107"/>
-      <c r="J19" s="107"/>
-      <c r="K19" s="107"/>
-      <c r="L19" s="107"/>
-      <c r="M19" s="107"/>
-      <c r="N19" s="107"/>
-      <c r="O19" s="107"/>
-    </row>
-    <row r="20" spans="1:15">
-      <c r="A20" s="107" t="s">
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="15"/>
+      <c r="K19" s="15"/>
+      <c r="L19" s="15"/>
+      <c r="M19" s="15"/>
+      <c r="N19" s="15"/>
+      <c r="O19" s="15"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A20" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="107"/>
-      <c r="C20" s="107"/>
-      <c r="D20" s="107"/>
-      <c r="E20" s="107"/>
-      <c r="F20" s="107"/>
-      <c r="G20" s="112"/>
-      <c r="H20" s="107"/>
-      <c r="I20" s="107"/>
-      <c r="J20" s="107"/>
-      <c r="K20" s="107"/>
-      <c r="L20" s="107"/>
-      <c r="M20" s="107"/>
-      <c r="N20" s="107"/>
-      <c r="O20" s="107"/>
-    </row>
-    <row r="21" spans="1:15">
-      <c r="A21" s="107" t="s">
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="15"/>
+      <c r="M20" s="15"/>
+      <c r="N20" s="15"/>
+      <c r="O20" s="15"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A21" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="B21" s="107"/>
-      <c r="C21" s="107"/>
-      <c r="D21" s="107"/>
-      <c r="E21" s="107"/>
-      <c r="F21" s="107"/>
-      <c r="G21" s="112"/>
-      <c r="H21" s="107"/>
-      <c r="I21" s="107"/>
-      <c r="J21" s="107"/>
-      <c r="K21" s="107"/>
-      <c r="L21" s="107"/>
-      <c r="M21" s="107"/>
-      <c r="N21" s="107"/>
-      <c r="O21" s="107"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="15"/>
+      <c r="J21" s="15"/>
+      <c r="K21" s="15"/>
+      <c r="L21" s="15"/>
+      <c r="M21" s="15"/>
+      <c r="N21" s="15"/>
+      <c r="O21" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="C1:C2"/>
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="H1:H2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="I1:L1"/>
     <mergeCell ref="M1:O1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="C1:C2"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <hyperlinks>
@@ -2636,725 +2588,750 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE4B6C87-4171-4F6D-A880-B7F7C78A6E37}">
   <dimension ref="B1:K42"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="14.28515625" customWidth="1"/>
-    <col min="3" max="3" width="13.140625" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" customWidth="1"/>
+    <col min="3" max="3" width="13.1640625" customWidth="1"/>
+    <col min="4" max="4" width="9.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" ht="15.75" thickBot="1"/>
-    <row r="2" spans="2:11" ht="26.25" thickBot="1">
-      <c r="B2" s="71" t="s">
+    <row r="1" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:11" ht="26" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="73"/>
-    </row>
-    <row r="3" spans="2:11" ht="18.75" thickBot="1">
-      <c r="B3" s="74" t="s">
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="32"/>
+    </row>
+    <row r="3" spans="2:11" ht="19" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="33" t="s">
         <v>131</v>
       </c>
-      <c r="C3" s="75"/>
-      <c r="D3" s="75"/>
-      <c r="E3" s="75"/>
-      <c r="F3" s="75"/>
-      <c r="G3" s="75"/>
-      <c r="H3" s="75"/>
-      <c r="I3" s="75"/>
-      <c r="J3" s="75"/>
-      <c r="K3" s="76"/>
-    </row>
-    <row r="4" spans="2:11" ht="15.75">
-      <c r="B4" s="44" t="s">
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="34"/>
+      <c r="I3" s="34"/>
+      <c r="J3" s="34"/>
+      <c r="K3" s="35"/>
+    </row>
+    <row r="4" spans="2:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="B4" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="77"/>
-      <c r="H4" s="78" t="s">
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="39" t="s">
         <v>48</v>
       </c>
-      <c r="I4" s="79"/>
-      <c r="J4" s="79"/>
-      <c r="K4" s="80"/>
-    </row>
-    <row r="5" spans="2:11">
-      <c r="B5" s="47" t="s">
+      <c r="I4" s="40"/>
+      <c r="J4" s="40"/>
+      <c r="K4" s="41"/>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B5" s="48" t="s">
         <v>49</v>
       </c>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="87" t="s">
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="50" t="s">
         <v>50</v>
       </c>
-      <c r="F5" s="87"/>
-      <c r="G5" s="88"/>
-      <c r="H5" s="81"/>
-      <c r="I5" s="82"/>
-      <c r="J5" s="82"/>
-      <c r="K5" s="83"/>
-    </row>
-    <row r="6" spans="2:11">
-      <c r="B6" s="89" t="s">
+      <c r="F5" s="50"/>
+      <c r="G5" s="51"/>
+      <c r="H5" s="42"/>
+      <c r="I5" s="43"/>
+      <c r="J5" s="43"/>
+      <c r="K5" s="44"/>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B6" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="90"/>
-      <c r="D6" s="90"/>
-      <c r="E6" s="91" t="s">
+      <c r="C6" s="53"/>
+      <c r="D6" s="53"/>
+      <c r="E6" s="54" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="92"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="81"/>
-      <c r="I6" s="82"/>
-      <c r="J6" s="82"/>
-      <c r="K6" s="83"/>
-    </row>
-    <row r="7" spans="2:11">
-      <c r="B7" s="94"/>
-      <c r="C7" s="95"/>
-      <c r="D7" s="95"/>
-      <c r="E7" s="95"/>
-      <c r="F7" s="95"/>
-      <c r="G7" s="96"/>
-      <c r="H7" s="81"/>
-      <c r="I7" s="82"/>
-      <c r="J7" s="82"/>
-      <c r="K7" s="83"/>
-    </row>
-    <row r="8" spans="2:11" ht="15.75">
-      <c r="B8" s="65" t="s">
+      <c r="F6" s="55"/>
+      <c r="G6" s="56"/>
+      <c r="H6" s="42"/>
+      <c r="I6" s="43"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="44"/>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B7" s="57"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="58"/>
+      <c r="F7" s="58"/>
+      <c r="G7" s="59"/>
+      <c r="H7" s="42"/>
+      <c r="I7" s="43"/>
+      <c r="J7" s="43"/>
+      <c r="K7" s="44"/>
+    </row>
+    <row r="8" spans="2:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="B8" s="60" t="s">
         <v>53</v>
       </c>
-      <c r="C8" s="66"/>
-      <c r="D8" s="66"/>
-      <c r="E8" s="66"/>
-      <c r="F8" s="66"/>
-      <c r="G8" s="97"/>
-      <c r="H8" s="81"/>
-      <c r="I8" s="82"/>
-      <c r="J8" s="82"/>
-      <c r="K8" s="83"/>
-    </row>
-    <row r="9" spans="2:11">
-      <c r="B9" s="98" t="s">
+      <c r="C8" s="61"/>
+      <c r="D8" s="61"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="61"/>
+      <c r="G8" s="62"/>
+      <c r="H8" s="42"/>
+      <c r="I8" s="43"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="44"/>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B9" s="63" t="s">
         <v>54</v>
       </c>
-      <c r="C9" s="99"/>
-      <c r="D9" s="99"/>
-      <c r="E9" s="99"/>
-      <c r="F9" s="99"/>
-      <c r="G9" s="100"/>
-      <c r="H9" s="81"/>
-      <c r="I9" s="82"/>
-      <c r="J9" s="82"/>
-      <c r="K9" s="83"/>
-    </row>
-    <row r="10" spans="2:11">
-      <c r="B10" s="101"/>
-      <c r="C10" s="102"/>
-      <c r="D10" s="102"/>
-      <c r="E10" s="102"/>
-      <c r="F10" s="102"/>
-      <c r="G10" s="103"/>
-      <c r="H10" s="81"/>
-      <c r="I10" s="82"/>
-      <c r="J10" s="82"/>
-      <c r="K10" s="83"/>
-    </row>
-    <row r="11" spans="2:11">
-      <c r="B11" s="101"/>
-      <c r="C11" s="102"/>
-      <c r="D11" s="102"/>
-      <c r="E11" s="102"/>
-      <c r="F11" s="102"/>
-      <c r="G11" s="103"/>
-      <c r="H11" s="81"/>
-      <c r="I11" s="82"/>
-      <c r="J11" s="82"/>
-      <c r="K11" s="83"/>
-    </row>
-    <row r="12" spans="2:11" ht="15.75" thickBot="1">
-      <c r="B12" s="104"/>
-      <c r="C12" s="105"/>
-      <c r="D12" s="105"/>
-      <c r="E12" s="105"/>
-      <c r="F12" s="105"/>
-      <c r="G12" s="106"/>
-      <c r="H12" s="84"/>
-      <c r="I12" s="85"/>
-      <c r="J12" s="85"/>
-      <c r="K12" s="86"/>
-    </row>
-    <row r="13" spans="2:11" ht="15.75">
-      <c r="B13" s="62"/>
-      <c r="C13" s="63"/>
-      <c r="D13" s="63"/>
-      <c r="E13" s="63"/>
-      <c r="F13" s="63"/>
-      <c r="G13" s="63"/>
-      <c r="H13" s="63"/>
-      <c r="I13" s="63"/>
-      <c r="J13" s="63"/>
-      <c r="K13" s="64"/>
-    </row>
-    <row r="14" spans="2:11" ht="15.75">
-      <c r="B14" s="65" t="s">
+      <c r="C9" s="64"/>
+      <c r="D9" s="64"/>
+      <c r="E9" s="64"/>
+      <c r="F9" s="64"/>
+      <c r="G9" s="65"/>
+      <c r="H9" s="42"/>
+      <c r="I9" s="43"/>
+      <c r="J9" s="43"/>
+      <c r="K9" s="44"/>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B10" s="66"/>
+      <c r="C10" s="67"/>
+      <c r="D10" s="67"/>
+      <c r="E10" s="67"/>
+      <c r="F10" s="67"/>
+      <c r="G10" s="68"/>
+      <c r="H10" s="42"/>
+      <c r="I10" s="43"/>
+      <c r="J10" s="43"/>
+      <c r="K10" s="44"/>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B11" s="66"/>
+      <c r="C11" s="67"/>
+      <c r="D11" s="67"/>
+      <c r="E11" s="67"/>
+      <c r="F11" s="67"/>
+      <c r="G11" s="68"/>
+      <c r="H11" s="42"/>
+      <c r="I11" s="43"/>
+      <c r="J11" s="43"/>
+      <c r="K11" s="44"/>
+    </row>
+    <row r="12" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="69"/>
+      <c r="C12" s="70"/>
+      <c r="D12" s="70"/>
+      <c r="E12" s="70"/>
+      <c r="F12" s="70"/>
+      <c r="G12" s="71"/>
+      <c r="H12" s="45"/>
+      <c r="I12" s="46"/>
+      <c r="J12" s="46"/>
+      <c r="K12" s="47"/>
+    </row>
+    <row r="13" spans="2:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="B13" s="72"/>
+      <c r="C13" s="73"/>
+      <c r="D13" s="73"/>
+      <c r="E13" s="73"/>
+      <c r="F13" s="73"/>
+      <c r="G13" s="73"/>
+      <c r="H13" s="73"/>
+      <c r="I13" s="73"/>
+      <c r="J13" s="73"/>
+      <c r="K13" s="74"/>
+    </row>
+    <row r="14" spans="2:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="B14" s="60" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="66"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="66"/>
-      <c r="F14" s="66"/>
-      <c r="G14" s="66"/>
-      <c r="H14" s="66"/>
-      <c r="I14" s="66"/>
-      <c r="J14" s="66"/>
-      <c r="K14" s="67"/>
-    </row>
-    <row r="15" spans="2:11" ht="15.75">
-      <c r="B15" s="58" t="s">
+      <c r="C14" s="61"/>
+      <c r="D14" s="61"/>
+      <c r="E14" s="61"/>
+      <c r="F14" s="61"/>
+      <c r="G14" s="61"/>
+      <c r="H14" s="61"/>
+      <c r="I14" s="61"/>
+      <c r="J14" s="61"/>
+      <c r="K14" s="75"/>
+    </row>
+    <row r="15" spans="2:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="B15" s="76" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="59"/>
-      <c r="D15" s="59"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="60"/>
-      <c r="G15" s="60"/>
-      <c r="H15" s="60"/>
-      <c r="I15" s="60"/>
-      <c r="J15" s="60"/>
-      <c r="K15" s="61"/>
-    </row>
-    <row r="16" spans="2:11">
-      <c r="B16" s="68" t="s">
+      <c r="C15" s="77"/>
+      <c r="D15" s="77"/>
+      <c r="E15" s="78"/>
+      <c r="F15" s="78"/>
+      <c r="G15" s="78"/>
+      <c r="H15" s="78"/>
+      <c r="I15" s="78"/>
+      <c r="J15" s="78"/>
+      <c r="K15" s="79"/>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B16" s="80" t="s">
         <v>57</v>
       </c>
-      <c r="C16" s="69"/>
-      <c r="D16" s="69" t="s">
+      <c r="C16" s="81"/>
+      <c r="D16" s="81" t="s">
         <v>58</v>
       </c>
-      <c r="E16" s="69"/>
-      <c r="F16" s="69" t="s">
+      <c r="E16" s="81"/>
+      <c r="F16" s="81" t="s">
         <v>59</v>
       </c>
-      <c r="G16" s="69"/>
-      <c r="H16" s="69" t="s">
+      <c r="G16" s="81"/>
+      <c r="H16" s="81" t="s">
         <v>60</v>
       </c>
-      <c r="I16" s="69"/>
-      <c r="J16" s="69" t="s">
+      <c r="I16" s="81"/>
+      <c r="J16" s="81" t="s">
         <v>61</v>
       </c>
-      <c r="K16" s="70"/>
-    </row>
-    <row r="17" spans="2:11">
-      <c r="B17" s="53" t="s">
+      <c r="K16" s="82"/>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B17" s="83" t="s">
         <v>62</v>
       </c>
-      <c r="C17" s="54"/>
-      <c r="D17" s="54" t="s">
+      <c r="C17" s="84"/>
+      <c r="D17" s="84" t="s">
         <v>63</v>
       </c>
-      <c r="E17" s="54"/>
-      <c r="F17" s="54">
+      <c r="E17" s="84"/>
+      <c r="F17" s="84">
         <v>12600</v>
       </c>
-      <c r="G17" s="54"/>
-      <c r="H17" s="54" t="s">
+      <c r="G17" s="84"/>
+      <c r="H17" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="I17" s="54"/>
-      <c r="J17" s="54">
+      <c r="I17" s="84"/>
+      <c r="J17" s="84">
         <v>1</v>
       </c>
-      <c r="K17" s="56"/>
-    </row>
-    <row r="18" spans="2:11">
-      <c r="B18" s="53" t="s">
+      <c r="K17" s="85"/>
+    </row>
+    <row r="18" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B18" s="83" t="s">
         <v>65</v>
       </c>
-      <c r="C18" s="54"/>
-      <c r="D18" s="54" t="s">
+      <c r="C18" s="84"/>
+      <c r="D18" s="84" t="s">
         <v>63</v>
       </c>
-      <c r="E18" s="54"/>
-      <c r="F18" s="54">
+      <c r="E18" s="84"/>
+      <c r="F18" s="84">
         <v>11400</v>
       </c>
-      <c r="G18" s="54"/>
-      <c r="H18" s="54" t="s">
+      <c r="G18" s="84"/>
+      <c r="H18" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="I18" s="54"/>
-      <c r="J18" s="54">
+      <c r="I18" s="84"/>
+      <c r="J18" s="84">
         <v>1</v>
       </c>
-      <c r="K18" s="56"/>
-    </row>
-    <row r="19" spans="2:11">
-      <c r="B19" s="53" t="s">
+      <c r="K18" s="85"/>
+    </row>
+    <row r="19" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B19" s="83" t="s">
         <v>66</v>
       </c>
-      <c r="C19" s="54"/>
-      <c r="D19" s="54" t="s">
+      <c r="C19" s="84"/>
+      <c r="D19" s="84" t="s">
         <v>63</v>
       </c>
-      <c r="E19" s="54"/>
-      <c r="F19" s="54">
+      <c r="E19" s="84"/>
+      <c r="F19" s="84">
         <v>40750</v>
       </c>
-      <c r="G19" s="54"/>
-      <c r="H19" s="54" t="s">
+      <c r="G19" s="84"/>
+      <c r="H19" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="I19" s="54"/>
-      <c r="J19" s="54">
+      <c r="I19" s="84"/>
+      <c r="J19" s="84">
         <v>1</v>
       </c>
-      <c r="K19" s="56"/>
-    </row>
-    <row r="20" spans="2:11">
-      <c r="B20" s="53" t="s">
+      <c r="K19" s="85"/>
+    </row>
+    <row r="20" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B20" s="83" t="s">
         <v>67</v>
       </c>
-      <c r="C20" s="54"/>
-      <c r="D20" s="54" t="s">
+      <c r="C20" s="84"/>
+      <c r="D20" s="84" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="54"/>
-      <c r="F20" s="54" t="s">
+      <c r="E20" s="84"/>
+      <c r="F20" s="84" t="s">
         <v>69</v>
       </c>
-      <c r="G20" s="54"/>
-      <c r="H20" s="54" t="s">
+      <c r="G20" s="84"/>
+      <c r="H20" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="I20" s="54"/>
-      <c r="J20" s="54">
+      <c r="I20" s="84"/>
+      <c r="J20" s="84">
         <v>5</v>
       </c>
-      <c r="K20" s="56"/>
-    </row>
-    <row r="21" spans="2:11" ht="15.75">
-      <c r="B21" s="58" t="s">
+      <c r="K20" s="85"/>
+    </row>
+    <row r="21" spans="2:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="B21" s="76" t="s">
         <v>70</v>
       </c>
-      <c r="C21" s="59"/>
-      <c r="D21" s="59"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="60"/>
-      <c r="G21" s="60"/>
-      <c r="H21" s="60"/>
-      <c r="I21" s="60"/>
-      <c r="J21" s="60"/>
-      <c r="K21" s="61"/>
-    </row>
-    <row r="22" spans="2:11">
-      <c r="B22" s="53" t="s">
+      <c r="C21" s="77"/>
+      <c r="D21" s="77"/>
+      <c r="E21" s="78"/>
+      <c r="F21" s="78"/>
+      <c r="G21" s="78"/>
+      <c r="H21" s="78"/>
+      <c r="I21" s="78"/>
+      <c r="J21" s="78"/>
+      <c r="K21" s="79"/>
+    </row>
+    <row r="22" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B22" s="83" t="s">
         <v>71</v>
       </c>
-      <c r="C22" s="54"/>
-      <c r="D22" s="54" t="s">
+      <c r="C22" s="84"/>
+      <c r="D22" s="84" t="s">
         <v>72</v>
       </c>
-      <c r="E22" s="54"/>
-      <c r="F22" s="57">
+      <c r="E22" s="84"/>
+      <c r="F22" s="86">
         <v>20</v>
       </c>
-      <c r="G22" s="57"/>
-      <c r="H22" s="54" t="s">
+      <c r="G22" s="86"/>
+      <c r="H22" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="I22" s="54"/>
-      <c r="J22" s="54"/>
-      <c r="K22" s="56"/>
-    </row>
-    <row r="23" spans="2:11">
-      <c r="B23" s="53" t="s">
+      <c r="I22" s="84"/>
+      <c r="J22" s="84"/>
+      <c r="K22" s="85"/>
+    </row>
+    <row r="23" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B23" s="83" t="s">
         <v>73</v>
       </c>
-      <c r="C23" s="54"/>
-      <c r="D23" s="54" t="s">
+      <c r="C23" s="84"/>
+      <c r="D23" s="84" t="s">
         <v>72</v>
       </c>
-      <c r="E23" s="54"/>
-      <c r="F23" s="57">
+      <c r="E23" s="84"/>
+      <c r="F23" s="86">
         <v>100</v>
       </c>
-      <c r="G23" s="57"/>
-      <c r="H23" s="54" t="s">
+      <c r="G23" s="86"/>
+      <c r="H23" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="I23" s="54"/>
-      <c r="J23" s="54"/>
-      <c r="K23" s="56"/>
-    </row>
-    <row r="24" spans="2:11">
-      <c r="B24" s="53" t="s">
+      <c r="I23" s="84"/>
+      <c r="J23" s="84"/>
+      <c r="K23" s="85"/>
+    </row>
+    <row r="24" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B24" s="83" t="s">
         <v>74</v>
       </c>
-      <c r="C24" s="54"/>
-      <c r="D24" s="54" t="s">
+      <c r="C24" s="84"/>
+      <c r="D24" s="84" t="s">
         <v>75</v>
       </c>
-      <c r="E24" s="54"/>
-      <c r="F24" s="57">
+      <c r="E24" s="84"/>
+      <c r="F24" s="86">
         <v>101325</v>
       </c>
-      <c r="G24" s="57"/>
-      <c r="H24" s="54" t="s">
+      <c r="G24" s="86"/>
+      <c r="H24" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="I24" s="54"/>
-      <c r="J24" s="54">
+      <c r="I24" s="84"/>
+      <c r="J24" s="84">
         <v>4</v>
       </c>
-      <c r="K24" s="56"/>
-    </row>
-    <row r="25" spans="2:11">
-      <c r="B25" s="53" t="s">
+      <c r="K24" s="85"/>
+    </row>
+    <row r="25" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B25" s="83" t="s">
         <v>76</v>
       </c>
-      <c r="C25" s="54"/>
-      <c r="D25" s="54" t="s">
+      <c r="C25" s="84"/>
+      <c r="D25" s="84" t="s">
         <v>63</v>
       </c>
-      <c r="E25" s="54"/>
-      <c r="F25" s="54">
+      <c r="E25" s="84"/>
+      <c r="F25" s="84">
         <v>40750</v>
       </c>
-      <c r="G25" s="54"/>
-      <c r="H25" s="54" t="s">
+      <c r="G25" s="84"/>
+      <c r="H25" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="I25" s="54"/>
-      <c r="J25" s="54" t="s">
+      <c r="I25" s="84"/>
+      <c r="J25" s="84" t="s">
         <v>77</v>
       </c>
-      <c r="K25" s="56"/>
-    </row>
-    <row r="26" spans="2:11">
-      <c r="B26" s="53" t="s">
+      <c r="K25" s="85"/>
+    </row>
+    <row r="26" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B26" s="83" t="s">
         <v>78</v>
       </c>
-      <c r="C26" s="54"/>
-      <c r="D26" s="54" t="s">
+      <c r="C26" s="84"/>
+      <c r="D26" s="84" t="s">
         <v>63</v>
       </c>
-      <c r="E26" s="54"/>
-      <c r="F26" s="54">
+      <c r="E26" s="84"/>
+      <c r="F26" s="84">
         <v>34000</v>
       </c>
-      <c r="G26" s="54"/>
-      <c r="H26" s="54" t="s">
+      <c r="G26" s="84"/>
+      <c r="H26" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="I26" s="54"/>
-      <c r="J26" s="54">
+      <c r="I26" s="84"/>
+      <c r="J26" s="84">
         <v>1</v>
       </c>
-      <c r="K26" s="56"/>
-    </row>
-    <row r="27" spans="2:11">
-      <c r="B27" s="53" t="s">
+      <c r="K26" s="85"/>
+    </row>
+    <row r="27" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B27" s="83" t="s">
         <v>79</v>
       </c>
-      <c r="C27" s="54"/>
-      <c r="D27" s="54" t="s">
+      <c r="C27" s="84"/>
+      <c r="D27" s="84" t="s">
         <v>68</v>
       </c>
-      <c r="E27" s="54"/>
-      <c r="F27" s="54">
+      <c r="E27" s="84"/>
+      <c r="F27" s="84">
         <v>2000</v>
       </c>
-      <c r="G27" s="54"/>
-      <c r="H27" s="54" t="s">
+      <c r="G27" s="84"/>
+      <c r="H27" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="I27" s="54"/>
-      <c r="J27" s="54">
+      <c r="I27" s="84"/>
+      <c r="J27" s="84">
         <v>3</v>
       </c>
-      <c r="K27" s="56"/>
-    </row>
-    <row r="28" spans="2:11">
-      <c r="B28" s="53" t="s">
+      <c r="K27" s="85"/>
+    </row>
+    <row r="28" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B28" s="83" t="s">
         <v>80</v>
       </c>
-      <c r="C28" s="54"/>
-      <c r="D28" s="54" t="s">
+      <c r="C28" s="84"/>
+      <c r="D28" s="84" t="s">
         <v>81</v>
       </c>
-      <c r="E28" s="54"/>
-      <c r="F28" s="54">
+      <c r="E28" s="84"/>
+      <c r="F28" s="84">
         <v>30</v>
       </c>
-      <c r="G28" s="54"/>
-      <c r="H28" s="54" t="s">
+      <c r="G28" s="84"/>
+      <c r="H28" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="I28" s="54"/>
-      <c r="J28" s="54">
+      <c r="I28" s="84"/>
+      <c r="J28" s="84">
         <v>5</v>
       </c>
-      <c r="K28" s="56"/>
-    </row>
-    <row r="29" spans="2:11">
-      <c r="B29" s="53" t="s">
+      <c r="K28" s="85"/>
+    </row>
+    <row r="29" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B29" s="83" t="s">
         <v>82</v>
       </c>
-      <c r="C29" s="54"/>
-      <c r="D29" s="54" t="s">
+      <c r="C29" s="84"/>
+      <c r="D29" s="84" t="s">
         <v>81</v>
       </c>
-      <c r="E29" s="54"/>
-      <c r="F29" s="55" t="s">
+      <c r="E29" s="84"/>
+      <c r="F29" s="95" t="s">
         <v>83</v>
       </c>
-      <c r="G29" s="55"/>
-      <c r="H29" s="54" t="s">
+      <c r="G29" s="95"/>
+      <c r="H29" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="I29" s="54"/>
-      <c r="J29" s="54">
+      <c r="I29" s="84"/>
+      <c r="J29" s="84">
         <v>5</v>
       </c>
-      <c r="K29" s="56"/>
-    </row>
-    <row r="30" spans="2:11">
-      <c r="B30" s="53" t="s">
+      <c r="K29" s="85"/>
+    </row>
+    <row r="30" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B30" s="83" t="s">
         <v>84</v>
       </c>
-      <c r="C30" s="54"/>
-      <c r="D30" s="54" t="s">
+      <c r="C30" s="84"/>
+      <c r="D30" s="84" t="s">
         <v>81</v>
       </c>
-      <c r="E30" s="54"/>
-      <c r="F30" s="55" t="s">
+      <c r="E30" s="84"/>
+      <c r="F30" s="95" t="s">
         <v>85</v>
       </c>
-      <c r="G30" s="55"/>
-      <c r="H30" s="54" t="s">
+      <c r="G30" s="95"/>
+      <c r="H30" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="I30" s="54"/>
-      <c r="J30" s="54">
+      <c r="I30" s="84"/>
+      <c r="J30" s="84">
         <v>5</v>
       </c>
-      <c r="K30" s="56"/>
-    </row>
-    <row r="31" spans="2:11">
-      <c r="B31" s="41"/>
-      <c r="C31" s="42"/>
-      <c r="D31" s="42"/>
-      <c r="E31" s="42"/>
-      <c r="F31" s="42"/>
-      <c r="G31" s="42"/>
-      <c r="H31" s="42"/>
-      <c r="I31" s="42"/>
-      <c r="J31" s="42"/>
-      <c r="K31" s="43"/>
-    </row>
-    <row r="32" spans="2:11" ht="15.75">
-      <c r="B32" s="44" t="s">
+      <c r="K30" s="85"/>
+    </row>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B31" s="87"/>
+      <c r="C31" s="88"/>
+      <c r="D31" s="88"/>
+      <c r="E31" s="88"/>
+      <c r="F31" s="88"/>
+      <c r="G31" s="88"/>
+      <c r="H31" s="88"/>
+      <c r="I31" s="88"/>
+      <c r="J31" s="88"/>
+      <c r="K31" s="89"/>
+    </row>
+    <row r="32" spans="2:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="B32" s="36" t="s">
         <v>86</v>
       </c>
-      <c r="C32" s="45"/>
-      <c r="D32" s="45"/>
-      <c r="E32" s="45"/>
-      <c r="F32" s="45"/>
-      <c r="G32" s="45"/>
-      <c r="H32" s="45"/>
-      <c r="I32" s="45"/>
-      <c r="J32" s="45"/>
-      <c r="K32" s="46"/>
-    </row>
-    <row r="33" spans="2:11">
-      <c r="B33" s="47" t="s">
+      <c r="C32" s="37"/>
+      <c r="D32" s="37"/>
+      <c r="E32" s="37"/>
+      <c r="F32" s="37"/>
+      <c r="G32" s="37"/>
+      <c r="H32" s="37"/>
+      <c r="I32" s="37"/>
+      <c r="J32" s="37"/>
+      <c r="K32" s="90"/>
+    </row>
+    <row r="33" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B33" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="C33" s="48"/>
-      <c r="D33" s="48"/>
-      <c r="E33" s="49" t="s">
+      <c r="C33" s="49"/>
+      <c r="D33" s="49"/>
+      <c r="E33" s="91" t="s">
         <v>88</v>
       </c>
-      <c r="F33" s="49"/>
-      <c r="G33" s="49"/>
-      <c r="H33" s="49"/>
-      <c r="I33" s="49"/>
-      <c r="J33" s="49"/>
-      <c r="K33" s="50"/>
-    </row>
-    <row r="34" spans="2:11">
-      <c r="B34" s="51" t="s">
+      <c r="F33" s="91"/>
+      <c r="G33" s="91"/>
+      <c r="H33" s="91"/>
+      <c r="I33" s="91"/>
+      <c r="J33" s="91"/>
+      <c r="K33" s="92"/>
+    </row>
+    <row r="34" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B34" s="93" t="s">
         <v>89</v>
       </c>
-      <c r="C34" s="52"/>
-      <c r="D34" s="52"/>
-      <c r="E34" s="49" t="s">
+      <c r="C34" s="94"/>
+      <c r="D34" s="94"/>
+      <c r="E34" s="91" t="s">
         <v>90</v>
       </c>
-      <c r="F34" s="49"/>
-      <c r="G34" s="49"/>
-      <c r="H34" s="49"/>
-      <c r="I34" s="49"/>
-      <c r="J34" s="49"/>
-      <c r="K34" s="50"/>
-    </row>
-    <row r="35" spans="2:11">
-      <c r="B35" s="24" t="s">
+      <c r="F34" s="91"/>
+      <c r="G34" s="91"/>
+      <c r="H34" s="91"/>
+      <c r="I34" s="91"/>
+      <c r="J34" s="91"/>
+      <c r="K34" s="92"/>
+    </row>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B35" s="105" t="s">
         <v>91</v>
       </c>
-      <c r="C35" s="25"/>
-      <c r="D35" s="25"/>
-      <c r="E35" s="28" t="s">
+      <c r="C35" s="106"/>
+      <c r="D35" s="106"/>
+      <c r="E35" s="109" t="s">
         <v>92</v>
       </c>
-      <c r="F35" s="28"/>
-      <c r="G35" s="28"/>
-      <c r="H35" s="28"/>
-      <c r="I35" s="28"/>
-      <c r="J35" s="28"/>
-      <c r="K35" s="29"/>
-    </row>
-    <row r="36" spans="2:11">
-      <c r="B36" s="26"/>
-      <c r="C36" s="27"/>
-      <c r="D36" s="27"/>
-      <c r="E36" s="30" t="s">
+      <c r="F35" s="109"/>
+      <c r="G35" s="109"/>
+      <c r="H35" s="109"/>
+      <c r="I35" s="109"/>
+      <c r="J35" s="109"/>
+      <c r="K35" s="110"/>
+    </row>
+    <row r="36" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B36" s="107"/>
+      <c r="C36" s="108"/>
+      <c r="D36" s="108"/>
+      <c r="E36" s="111" t="s">
         <v>93</v>
       </c>
-      <c r="F36" s="30"/>
-      <c r="G36" s="30"/>
-      <c r="H36" s="30"/>
-      <c r="I36" s="30"/>
-      <c r="J36" s="30"/>
-      <c r="K36" s="31"/>
-    </row>
-    <row r="37" spans="2:11" ht="15.75">
-      <c r="B37" s="32" t="s">
+      <c r="F36" s="111"/>
+      <c r="G36" s="111"/>
+      <c r="H36" s="111"/>
+      <c r="I36" s="111"/>
+      <c r="J36" s="111"/>
+      <c r="K36" s="112"/>
+    </row>
+    <row r="37" spans="2:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="B37" s="113" t="s">
         <v>61</v>
       </c>
-      <c r="C37" s="33"/>
-      <c r="D37" s="33"/>
-      <c r="E37" s="33"/>
-      <c r="F37" s="33"/>
-      <c r="G37" s="33"/>
-      <c r="H37" s="33"/>
-      <c r="I37" s="33"/>
-      <c r="J37" s="33"/>
-      <c r="K37" s="34"/>
-    </row>
-    <row r="38" spans="2:11" ht="145.5" customHeight="1">
-      <c r="B38" s="35" t="s">
+      <c r="C37" s="114"/>
+      <c r="D37" s="114"/>
+      <c r="E37" s="114"/>
+      <c r="F37" s="114"/>
+      <c r="G37" s="114"/>
+      <c r="H37" s="114"/>
+      <c r="I37" s="114"/>
+      <c r="J37" s="114"/>
+      <c r="K37" s="115"/>
+    </row>
+    <row r="38" spans="2:11" ht="145.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B38" s="116" t="s">
         <v>94</v>
       </c>
-      <c r="C38" s="36"/>
-      <c r="D38" s="36"/>
-      <c r="E38" s="36"/>
-      <c r="F38" s="36"/>
-      <c r="G38" s="36"/>
-      <c r="H38" s="36"/>
-      <c r="I38" s="36"/>
-      <c r="J38" s="36"/>
-      <c r="K38" s="37"/>
-    </row>
-    <row r="39" spans="2:11">
-      <c r="B39" s="38"/>
-      <c r="C39" s="39"/>
-      <c r="D39" s="39"/>
-      <c r="E39" s="39"/>
-      <c r="F39" s="39"/>
-      <c r="G39" s="39"/>
-      <c r="H39" s="39"/>
-      <c r="I39" s="39"/>
-      <c r="J39" s="39"/>
-      <c r="K39" s="40"/>
-    </row>
-    <row r="40" spans="2:11" ht="15.75">
-      <c r="B40" s="15" t="s">
+      <c r="C38" s="117"/>
+      <c r="D38" s="117"/>
+      <c r="E38" s="117"/>
+      <c r="F38" s="117"/>
+      <c r="G38" s="117"/>
+      <c r="H38" s="117"/>
+      <c r="I38" s="117"/>
+      <c r="J38" s="117"/>
+      <c r="K38" s="118"/>
+    </row>
+    <row r="39" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B39" s="119"/>
+      <c r="C39" s="120"/>
+      <c r="D39" s="120"/>
+      <c r="E39" s="120"/>
+      <c r="F39" s="120"/>
+      <c r="G39" s="120"/>
+      <c r="H39" s="120"/>
+      <c r="I39" s="120"/>
+      <c r="J39" s="120"/>
+      <c r="K39" s="121"/>
+    </row>
+    <row r="40" spans="2:11" ht="16" x14ac:dyDescent="0.2">
+      <c r="B40" s="96" t="s">
         <v>95</v>
       </c>
-      <c r="C40" s="16"/>
-      <c r="D40" s="16"/>
-      <c r="E40" s="16"/>
-      <c r="F40" s="16"/>
-      <c r="G40" s="16"/>
-      <c r="H40" s="16"/>
-      <c r="I40" s="16"/>
-      <c r="J40" s="16"/>
-      <c r="K40" s="17"/>
-    </row>
-    <row r="41" spans="2:11">
-      <c r="B41" s="18" t="s">
+      <c r="C40" s="97"/>
+      <c r="D40" s="97"/>
+      <c r="E40" s="97"/>
+      <c r="F40" s="97"/>
+      <c r="G40" s="97"/>
+      <c r="H40" s="97"/>
+      <c r="I40" s="97"/>
+      <c r="J40" s="97"/>
+      <c r="K40" s="98"/>
+    </row>
+    <row r="41" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B41" s="99" t="s">
         <v>96</v>
       </c>
-      <c r="C41" s="19"/>
-      <c r="D41" s="19"/>
-      <c r="E41" s="19"/>
-      <c r="F41" s="19"/>
-      <c r="G41" s="19"/>
-      <c r="H41" s="19"/>
-      <c r="I41" s="19"/>
-      <c r="J41" s="19"/>
-      <c r="K41" s="20"/>
-    </row>
-    <row r="42" spans="2:11" ht="15.75" thickBot="1">
-      <c r="B42" s="21"/>
-      <c r="C42" s="22"/>
-      <c r="D42" s="22"/>
-      <c r="E42" s="22"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="22"/>
-      <c r="H42" s="22"/>
-      <c r="I42" s="22"/>
-      <c r="J42" s="22"/>
-      <c r="K42" s="23"/>
+      <c r="C41" s="100"/>
+      <c r="D41" s="100"/>
+      <c r="E41" s="100"/>
+      <c r="F41" s="100"/>
+      <c r="G41" s="100"/>
+      <c r="H41" s="100"/>
+      <c r="I41" s="100"/>
+      <c r="J41" s="100"/>
+      <c r="K41" s="101"/>
+    </row>
+    <row r="42" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="102"/>
+      <c r="C42" s="103"/>
+      <c r="D42" s="103"/>
+      <c r="E42" s="103"/>
+      <c r="F42" s="103"/>
+      <c r="G42" s="103"/>
+      <c r="H42" s="103"/>
+      <c r="I42" s="103"/>
+      <c r="J42" s="103"/>
+      <c r="K42" s="104"/>
     </row>
   </sheetData>
   <mergeCells count="102">
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="H4:K12"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="B9:G12"/>
-    <mergeCell ref="B13:K13"/>
-    <mergeCell ref="B14:K14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="E15:K15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="B40:K40"/>
+    <mergeCell ref="B41:K41"/>
+    <mergeCell ref="B42:K42"/>
+    <mergeCell ref="B35:D36"/>
+    <mergeCell ref="E35:K35"/>
+    <mergeCell ref="E36:K36"/>
+    <mergeCell ref="B37:K37"/>
+    <mergeCell ref="B38:K38"/>
+    <mergeCell ref="B39:K39"/>
+    <mergeCell ref="B31:K31"/>
+    <mergeCell ref="B32:K32"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="E33:K33"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="E34:K34"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="J24:K24"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="E21:K21"/>
     <mergeCell ref="B22:C22"/>
@@ -3372,61 +3349,36 @@
     <mergeCell ref="F20:G20"/>
     <mergeCell ref="H20:I20"/>
     <mergeCell ref="J20:K20"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="H28:I28"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="B31:K31"/>
-    <mergeCell ref="B32:K32"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="E33:K33"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="E34:K34"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="B40:K40"/>
-    <mergeCell ref="B41:K41"/>
-    <mergeCell ref="B42:K42"/>
-    <mergeCell ref="B35:D36"/>
-    <mergeCell ref="E35:K35"/>
-    <mergeCell ref="E36:K36"/>
-    <mergeCell ref="B37:K37"/>
-    <mergeCell ref="B38:K38"/>
-    <mergeCell ref="B39:K39"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="B13:K13"/>
+    <mergeCell ref="B14:K14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="E15:K15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="H4:K12"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B9:G12"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <hyperlinks>
@@ -3434,22 +3386,21 @@
     <hyperlink ref="E35:K35" r:id="rId2" location=":~:text=Polar%20cranes%20operate%20on%20a,as%20during%20the%20refuelling%20outages." display="Nuclear Polar Crane Product" xr:uid="{F03E8A74-7D8A-47F5-AEDC-693557EEC008}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{638A591F-E9F2-410B-B046-D77C1ADE1A9B}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" customWidth="1"/>
-    <col min="2" max="2" width="5.7109375" customWidth="1"/>
-    <col min="3" max="3" width="70.42578125" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" customWidth="1"/>
+    <col min="3" max="3" width="70.5" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="20.100000000000001" customHeight="1">
+    <row r="1" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>97</v>
       </c>
@@ -3457,7 +3408,7 @@
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -3471,7 +3422,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -3485,7 +3436,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -3499,7 +3450,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -3513,7 +3464,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -3527,7 +3478,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -3537,17 +3488,17 @@
       <c r="C7" s="8"/>
       <c r="D7" s="7"/>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>19</v>
       </c>
@@ -3561,21 +3512,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C335437-7450-407F-A883-DAB44B3984CA}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" customWidth="1"/>
-    <col min="2" max="2" width="5.7109375" customWidth="1"/>
-    <col min="3" max="3" width="68.5703125" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" customWidth="1"/>
+    <col min="3" max="3" width="68.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="11" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1">
+    <row r="1" spans="1:3" s="11" customFormat="1" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="9" t="s">
         <v>112</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="10"/>
     </row>
-    <row r="2" spans="1:3" s="14" customFormat="1" ht="15" customHeight="1" thickBot="1">
+    <row r="2" spans="1:3" s="14" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
         <v>1</v>
       </c>
@@ -3586,7 +3537,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -3597,7 +3548,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -3608,7 +3559,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -3619,7 +3570,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -3630,7 +3581,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -3641,7 +3592,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -3652,7 +3603,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
@@ -3663,7 +3614,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -3674,7 +3625,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -3685,7 +3636,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -3693,27 +3644,27 @@
         <v>128</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:1">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>19</v>
       </c>
@@ -3727,32 +3678,32 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CFA08BB-FCE4-4222-8A52-F77A6275FA26}">
   <dimension ref="B2:B6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="2:2">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="2:2">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="2:2">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="2:2">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>5</v>
       </c>
@@ -3764,6 +3715,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CDA27708AEC7164FA5A8E7F34BA13E1C" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d337e44b8df9141dd8e32c49a28cd2a0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8c45fcf1-ee50-4456-b421-c5762743e248" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bceaae793d8b2739ec45359ab7106e71" ns2:_="">
     <xsd:import namespace="8c45fcf1-ee50-4456-b421-c5762743e248"/>
@@ -3931,12 +3888,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -3947,6 +3898,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2270B468-AF36-4411-AF0D-A5972E279566}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="1fe95263-70f5-4c95-8f03-1a74b2e094c7"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="f763a930-6dc6-48d0-9234-549914b51acc"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1606E962-CB6D-4D64-B073-D0E05B28D5E7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3964,23 +3932,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2270B468-AF36-4411-AF0D-A5972E279566}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="1fe95263-70f5-4c95-8f03-1a74b2e094c7"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="f763a930-6dc6-48d0-9234-549914b51acc"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E3BC41F-1913-4E04-909D-E64B0BFBFB5B}">
   <ds:schemaRefs>

</xml_diff>